<commit_message>
Fix typo in fetch_data instructions
</commit_message>
<xml_diff>
--- a/processed-data/19_data_uploads/03_manifest/manifest_open.xlsx
+++ b/processed-data/19_data_uploads/03_manifest/manifest_open.xlsx
@@ -716,7 +716,7 @@
     <t xml:space="preserve">75e265f618b0d50aba88f78c5acf6a8b</t>
   </si>
   <si>
-    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('HD_spe_cell') from spatialLIBD &gt;= 1.25.5.</t>
+    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('habenula_atlas_HD_spe_cell') from spatialLIBD &gt;= 1.25.5.</t>
   </si>
   <si>
     <t xml:space="preserve">habenula_atlas_HD_spe_cell_pseudobulk.rds</t>
@@ -725,7 +725,7 @@
     <t xml:space="preserve">22ebb432a48cb6f85c6f05063f984f7c</t>
   </si>
   <si>
-    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('HD_spe_cell_pseudobulk') from spatialLIBD &gt;= 1.25.5.</t>
+    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('habenula_atlas_HD_spe_cell_pseudobulk') from spatialLIBD &gt;= 1.25.5.</t>
   </si>
   <si>
     <t xml:space="preserve">habenula_atlas_visium_spe.rds</t>
@@ -734,7 +734,7 @@
     <t xml:space="preserve">64ce6ae9151c71717bfb169f21d73f32</t>
   </si>
   <si>
-    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('visium_spe') from spatialLIBD &gt;= 1.25.5.</t>
+    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('habenula_atlas_visium_spe') from spatialLIBD &gt;= 1.25.5.</t>
   </si>
   <si>
     <t xml:space="preserve">habenula_atlas_visium_spe_pseudobulk.rds</t>
@@ -743,7 +743,7 @@
     <t xml:space="preserve">d2893cd456f38bbeeb3ebd0b88e8585b</t>
   </si>
   <si>
-    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('visium_spe_pseudobulk') from spatialLIBD &gt;= 1.25.5.</t>
+    <t xml:space="preserve">R object is a SpatialExperiment (v1.18.1) and can alternatively be retrieved with spatialLIBD::fetch_data('habenula_atlas_visium_spe_pseudobulk') from spatialLIBD &gt;= 1.25.5.</t>
   </si>
   <si>
     <t xml:space="preserve">habenula_atlas_snMultiome_seurat_cell.rds</t>
@@ -752,7 +752,7 @@
     <t xml:space="preserve">feb5a2d65918fd3f7b46391e0155cbc9</t>
   </si>
   <si>
-    <t xml:space="preserve">R object is a Seurat (v5.3.0) object and can alternatively be retrieved with spatialLIBD::fetch_data('snMultiome_seurat_cell') from spatialLIBD &gt;= 1.25.5.</t>
+    <t xml:space="preserve">R object is a Seurat (v5.3.0) object and can alternatively be retrieved with spatialLIBD::fetch_data('habenula_atlas_snMultiome_seurat_cell') from spatialLIBD &gt;= 1.25.5.</t>
   </si>
   <si>
     <t xml:space="preserve">habenula_atlas_snMultiome_seurat_metacell.rds</t>
@@ -761,7 +761,7 @@
     <t xml:space="preserve">1bcb148edbd12085bd41358b5cfd6fee</t>
   </si>
   <si>
-    <t xml:space="preserve">R object is a Seurat (v5.3.0) object and can alternatively be retrieved with spatialLIBD::fetch_data('snMultiome_seurat_metacell') from spatialLIBD &gt;= 1.25.5.</t>
+    <t xml:space="preserve">R object is a Seurat (v5.3.0) object and can alternatively be retrieved with spatialLIBD::fetch_data('habenula_atlas_snMultiome_seurat_metacell') from spatialLIBD &gt;= 1.25.5.</t>
   </si>
   <si>
     <t xml:space="preserve">Br3942_barcodes.tsv.gz</t>

</xml_diff>